<commit_message>
added in looping for parsing data in xml files
</commit_message>
<xml_diff>
--- a/parsedData.xlsx
+++ b/parsedData.xlsx
@@ -413,9 +413,214 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>yahoo.com</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>dmarc@yahoo.com</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>zyx987654</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>yahoo.com</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>dmarc@yahoo.com</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>zyx987654</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>yahoo.com</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>dmarc@yahoo.com</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>zyx987654</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>yahoo.com</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>dmarc@yahoo.com</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>zyx987654</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>outlook.com</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>dmarc@outlook.com</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>abcdef12345</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>outlook.com</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>dmarc@outlook.com</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>abcdef12345</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>outlook.com</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>dmarc@outlook.com</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>abcdef12345</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>outlook.com</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>dmarc@outlook.com</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>abcdef12345</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>google.com</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>noreply-dmarc-support@google.com</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>1234567890</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>google.com</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>noreply-dmarc-support@google.com</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>1234567890</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>google.com</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>noreply-dmarc-support@google.com</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>1234567890</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>google.com</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>noreply-dmarc-support@google.com</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>1234567890</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>